<commit_message>
Lab 4 fixes: thousands axis format in scenario chart, left aligned workbook check cell
</commit_message>
<xml_diff>
--- a/lab4/out/lab4_pricing.xlsx
+++ b/lab4/out/lab4_pricing.xlsx
@@ -126,7 +126,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
@@ -144,12 +144,15 @@
       <alignment horizontal="right" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="top" wrapText="1"/>
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="4" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -401,6 +404,7 @@
             </rich>
           </tx>
         </title>
+        <numFmt formatCode="#,##0" sourceLinked="0"/>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="10"/>
@@ -1786,7 +1790,7 @@
         <f>AVERAGE(C2:G2)</f>
         <v/>
       </c>
-      <c r="I2" s="6">
+      <c r="I2" s="9">
         <f>RANK(H2,$H$2:$H$4)</f>
         <v/>
       </c>
@@ -1821,7 +1825,7 @@
         <f>AVERAGE(C3:G3)</f>
         <v/>
       </c>
-      <c r="I3" s="6">
+      <c r="I3" s="9">
         <f>RANK(H3,$H$2:$H$4)</f>
         <v/>
       </c>
@@ -1856,7 +1860,7 @@
         <f>AVERAGE(C4:G4)</f>
         <v/>
       </c>
-      <c r="I4" s="6">
+      <c r="I4" s="9">
         <f>RANK(H4,$H$2:$H$4)</f>
         <v/>
       </c>
@@ -1921,13 +1925,13 @@
           <t>вхід</t>
         </is>
       </c>
-      <c r="C2" s="9" t="n">
+      <c r="C2" s="10" t="n">
         <v>25</v>
       </c>
-      <c r="D2" s="9" t="n">
+      <c r="D2" s="10" t="n">
         <v>50</v>
       </c>
-      <c r="E2" s="9" t="n">
+      <c r="E2" s="10" t="n">
         <v>150</v>
       </c>
     </row>
@@ -1942,13 +1946,13 @@
           <t>вхід</t>
         </is>
       </c>
-      <c r="C3" s="9" t="n">
+      <c r="C3" s="10" t="n">
         <v>110</v>
       </c>
-      <c r="D3" s="9" t="n">
+      <c r="D3" s="10" t="n">
         <v>110</v>
       </c>
-      <c r="E3" s="9" t="n">
+      <c r="E3" s="10" t="n">
         <v>90</v>
       </c>
     </row>
@@ -1963,13 +1967,13 @@
           <t>захисне правило</t>
         </is>
       </c>
-      <c r="C4" s="10" t="n">
+      <c r="C4" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="D4" s="10" t="n">
+      <c r="D4" s="11" t="n">
         <v>5</v>
       </c>
-      <c r="E4" s="10" t="n">
+      <c r="E4" s="11" t="n">
         <v>20</v>
       </c>
     </row>
@@ -1984,13 +1988,13 @@
           <t>A1</t>
         </is>
       </c>
-      <c r="C5" s="11" t="n">
+      <c r="C5" s="12" t="n">
         <v>0.6</v>
       </c>
-      <c r="D5" s="11" t="n">
+      <c r="D5" s="12" t="n">
         <v>0.3</v>
       </c>
-      <c r="E5" s="11" t="n">
+      <c r="E5" s="12" t="n">
         <v>0.1</v>
       </c>
     </row>
@@ -2005,13 +2009,13 @@
           <t>A2</t>
         </is>
       </c>
-      <c r="C6" s="12" t="n">
+      <c r="C6" s="13" t="n">
         <v>1</v>
       </c>
-      <c r="D6" s="12" t="n">
+      <c r="D6" s="13" t="n">
         <v>2</v>
       </c>
-      <c r="E6" s="12" t="n">
+      <c r="E6" s="13" t="n">
         <v>5</v>
       </c>
     </row>
@@ -2047,15 +2051,15 @@
           <t>год × 30</t>
         </is>
       </c>
-      <c r="C8" s="13">
+      <c r="C8" s="14">
         <f>C7*x4_sup_rate</f>
         <v/>
       </c>
-      <c r="D8" s="13">
+      <c r="D8" s="14">
         <f>D7*x4_sup_rate</f>
         <v/>
       </c>
-      <c r="E8" s="13">
+      <c r="E8" s="14">
         <f>E7*x4_sup_rate</f>
         <v/>
       </c>
@@ -2071,15 +2075,15 @@
           <t>база + ціна × usage</t>
         </is>
       </c>
-      <c r="C9" s="13">
+      <c r="C9" s="14">
         <f>C2+C3*C6</f>
         <v/>
       </c>
-      <c r="D9" s="13">
+      <c r="D9" s="14">
         <f>D2+D3*D6</f>
         <v/>
       </c>
-      <c r="E9" s="13">
+      <c r="E9" s="14">
         <f>E2+E3*E6</f>
         <v/>
       </c>
@@ -2095,15 +2099,15 @@
           <t>COGS бази + usage × 16</t>
         </is>
       </c>
-      <c r="C10" s="13">
+      <c r="C10" s="14">
         <f>C8+C6*x4_cogs</f>
         <v/>
       </c>
-      <c r="D10" s="13">
+      <c r="D10" s="14">
         <f>D8+D6*x4_cogs</f>
         <v/>
       </c>
-      <c r="E10" s="13">
+      <c r="E10" s="14">
         <f>E8+E6*x4_cogs</f>
         <v/>
       </c>
@@ -2119,15 +2123,15 @@
           <t>рахунок мінус COGS</t>
         </is>
       </c>
-      <c r="C11" s="13">
+      <c r="C11" s="14">
         <f>C9-C10</f>
         <v/>
       </c>
-      <c r="D11" s="13">
+      <c r="D11" s="14">
         <f>D9-D10</f>
         <v/>
       </c>
-      <c r="E11" s="13">
+      <c r="E11" s="14">
         <f>E9-E10</f>
         <v/>
       </c>
@@ -2143,15 +2147,15 @@
           <t>(Revenue − COGS) / Revenue</t>
         </is>
       </c>
-      <c r="C12" s="14">
+      <c r="C12" s="15">
         <f>(C9-C10)/C9</f>
         <v/>
       </c>
-      <c r="D12" s="14">
+      <c r="D12" s="15">
         <f>(D9-D10)/D9</f>
         <v/>
       </c>
-      <c r="E12" s="14">
+      <c r="E12" s="15">
         <f>(E9-E10)/E9</f>
         <v/>
       </c>
@@ -2167,15 +2171,15 @@
           <t>COGS / (1 − 0,70)</t>
         </is>
       </c>
-      <c r="C13" s="13">
+      <c r="C13" s="14">
         <f>C10/(1-x4_gm)</f>
         <v/>
       </c>
-      <c r="D13" s="13">
+      <c r="D13" s="14">
         <f>D10/(1-x4_gm)</f>
         <v/>
       </c>
-      <c r="E13" s="13">
+      <c r="E13" s="14">
         <f>E10/(1-x4_gm)</f>
         <v/>
       </c>
@@ -2191,15 +2195,15 @@
           <t>порівняння</t>
         </is>
       </c>
-      <c r="C14" s="13">
+      <c r="C14" s="14">
         <f>IF(C9&gt;=C13,"так","ні")</f>
         <v/>
       </c>
-      <c r="D14" s="13">
+      <c r="D14" s="14">
         <f>IF(D9&gt;=D13,"так","ні")</f>
         <v/>
       </c>
-      <c r="E14" s="13">
+      <c r="E14" s="14">
         <f>IF(E9&gt;=E13,"так","ні")</f>
         <v/>
       </c>
@@ -2215,15 +2219,15 @@
           <t>(ціна − COGS) / COGS</t>
         </is>
       </c>
-      <c r="C15" s="14">
+      <c r="C15" s="15">
         <f>(C9-C10)/C10</f>
         <v/>
       </c>
-      <c r="D15" s="14">
+      <c r="D15" s="15">
         <f>(D9-D10)/D10</f>
         <v/>
       </c>
-      <c r="E15" s="14">
+      <c r="E15" s="15">
         <f>(E9-E10)/E10</f>
         <v/>
       </c>
@@ -2239,15 +2243,15 @@
           <t>рахунок / usage</t>
         </is>
       </c>
-      <c r="C16" s="13">
+      <c r="C16" s="14">
         <f>C9/C6</f>
         <v/>
       </c>
-      <c r="D16" s="13">
+      <c r="D16" s="14">
         <f>D9/D6</f>
         <v/>
       </c>
-      <c r="E16" s="13">
+      <c r="E16" s="14">
         <f>E9/E6</f>
         <v/>
       </c>
@@ -2263,15 +2267,15 @@
           <t>ціна будівлі / цінність</t>
         </is>
       </c>
-      <c r="C17" s="14">
+      <c r="C17" s="15">
         <f>C16/x4_value</f>
         <v/>
       </c>
-      <c r="D17" s="14">
+      <c r="D17" s="15">
         <f>D16/x4_value</f>
         <v/>
       </c>
-      <c r="E17" s="14">
+      <c r="E17" s="15">
         <f>E16/x4_value</f>
         <v/>
       </c>
@@ -2287,15 +2291,15 @@
           <t>ціна будівлі ≥ 53,33</t>
         </is>
       </c>
-      <c r="C18" s="13">
+      <c r="C18" s="14">
         <f>IF(C3&gt;=x4_floor_unit,"так","ні")</f>
         <v/>
       </c>
-      <c r="D18" s="13">
+      <c r="D18" s="14">
         <f>IF(D3&gt;=x4_floor_unit,"так","ні")</f>
         <v/>
       </c>
-      <c r="E18" s="13">
+      <c r="E18" s="14">
         <f>IF(E3&gt;=x4_floor_unit,"так","ні")</f>
         <v/>
       </c>
@@ -2311,15 +2315,15 @@
           <t>COGS бази / COGS клієнта</t>
         </is>
       </c>
-      <c r="C19" s="14">
+      <c r="C19" s="15">
         <f>C8/C10</f>
         <v/>
       </c>
-      <c r="D19" s="14">
+      <c r="D19" s="15">
         <f>D8/D10</f>
         <v/>
       </c>
-      <c r="E19" s="14">
+      <c r="E19" s="15">
         <f>E8/E10</f>
         <v/>
       </c>
@@ -2351,7 +2355,7 @@
         <f>x4_cogs_var/(1-x4_gm)</f>
         <v/>
       </c>
-      <c r="C22" s="14">
+      <c r="C22" s="15">
         <f>(B22-x4_cogs_var)/B22</f>
         <v/>
       </c>
@@ -2366,7 +2370,7 @@
         <f>x4_cogs_var*(1+x4_gm)</f>
         <v/>
       </c>
-      <c r="C23" s="14">
+      <c r="C23" s="15">
         <f>(B23-x4_cogs_var)/B23</f>
         <v/>
       </c>
@@ -2431,13 +2435,13 @@
           <t>максимум тарифу</t>
         </is>
       </c>
-      <c r="C2" s="10" t="n">
+      <c r="C2" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="D2" s="10" t="n">
+      <c r="D2" s="11" t="n">
         <v>5</v>
       </c>
-      <c r="E2" s="10" t="n">
+      <c r="E2" s="11" t="n">
         <v>20</v>
       </c>
     </row>
@@ -2452,15 +2456,15 @@
           <t>база + ціна × n</t>
         </is>
       </c>
-      <c r="C3" s="13">
+      <c r="C3" s="14">
         <f>'Тарифи'!C2+'Тарифи'!C3*C2</f>
         <v/>
       </c>
-      <c r="D3" s="13">
+      <c r="D3" s="14">
         <f>'Тарифи'!D2+'Тарифи'!D3*D2</f>
         <v/>
       </c>
-      <c r="E3" s="13">
+      <c r="E3" s="14">
         <f>'Тарифи'!E2+'Тарифи'!E3*E2</f>
         <v/>
       </c>
@@ -2476,15 +2480,15 @@
           <t>COGS бази + n × COGS high</t>
         </is>
       </c>
-      <c r="C4" s="13">
+      <c r="C4" s="14">
         <f>'Тарифи'!C8+C2*x4_cogs_high</f>
         <v/>
       </c>
-      <c r="D4" s="13">
+      <c r="D4" s="14">
         <f>'Тарифи'!D8+D2*x4_cogs_high</f>
         <v/>
       </c>
-      <c r="E4" s="13">
+      <c r="E4" s="14">
         <f>'Тарифи'!E8+E2*x4_cogs_high</f>
         <v/>
       </c>
@@ -2496,15 +2500,15 @@
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr"/>
-      <c r="C5" s="14">
+      <c r="C5" s="15">
         <f>(C3-C4)/C3</f>
         <v/>
       </c>
-      <c r="D5" s="14">
+      <c r="D5" s="15">
         <f>(D3-D4)/D3</f>
         <v/>
       </c>
-      <c r="E5" s="14">
+      <c r="E5" s="15">
         <f>(E3-E4)/E3</f>
         <v/>
       </c>
@@ -2520,15 +2524,15 @@
           <t>n × (доплата + SMS)</t>
         </is>
       </c>
-      <c r="C6" s="13">
+      <c r="C6" s="14">
         <f>C2*x4_over</f>
         <v/>
       </c>
-      <c r="D6" s="13">
+      <c r="D6" s="14">
         <f>D2*x4_over</f>
         <v/>
       </c>
-      <c r="E6" s="13">
+      <c r="E6" s="14">
         <f>E2*x4_over</f>
         <v/>
       </c>
@@ -2540,15 +2544,15 @@
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr"/>
-      <c r="C7" s="13">
+      <c r="C7" s="14">
         <f>C3+C6</f>
         <v/>
       </c>
-      <c r="D7" s="13">
+      <c r="D7" s="14">
         <f>D3+D6</f>
         <v/>
       </c>
-      <c r="E7" s="13">
+      <c r="E7" s="14">
         <f>E3+E6</f>
         <v/>
       </c>
@@ -2560,15 +2564,15 @@
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr"/>
-      <c r="C8" s="14">
+      <c r="C8" s="15">
         <f>(C7-C4)/C7</f>
         <v/>
       </c>
-      <c r="D8" s="14">
+      <c r="D8" s="15">
         <f>(D7-D4)/D7</f>
         <v/>
       </c>
-      <c r="E8" s="14">
+      <c r="E8" s="15">
         <f>(E7-E4)/E7</f>
         <v/>
       </c>
@@ -2580,15 +2584,15 @@
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr"/>
-      <c r="C9" s="13">
+      <c r="C9" s="14">
         <f>IF(C5&gt;=x4_gm,"так","ні")</f>
         <v/>
       </c>
-      <c r="D9" s="13">
+      <c r="D9" s="14">
         <f>IF(D5&gt;=x4_gm,"так","ні")</f>
         <v/>
       </c>
-      <c r="E9" s="13">
+      <c r="E9" s="14">
         <f>IF(E5&gt;=x4_gm,"так","ні")</f>
         <v/>
       </c>
@@ -2600,15 +2604,15 @@
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr"/>
-      <c r="C10" s="13">
+      <c r="C10" s="14">
         <f>IF(C8&gt;=x4_gm,"так","ні")</f>
         <v/>
       </c>
-      <c r="D10" s="13">
+      <c r="D10" s="14">
         <f>IF(D8&gt;=x4_gm,"так","ні")</f>
         <v/>
       </c>
-      <c r="E10" s="13">
+      <c r="E10" s="14">
         <f>IF(E8&gt;=x4_gm,"так","ні")</f>
         <v/>
       </c>
@@ -2662,13 +2666,13 @@
           <t>Коефіцієнт масштабу</t>
         </is>
       </c>
-      <c r="B2" s="15" t="n">
+      <c r="B2" s="16" t="n">
         <v>0.7</v>
       </c>
-      <c r="C2" s="15" t="n">
+      <c r="C2" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D2" s="15" t="n">
+      <c r="D2" s="16" t="n">
         <v>1.4</v>
       </c>
     </row>
@@ -2678,15 +2682,15 @@
           <t>Платні будівлі (billable units)</t>
         </is>
       </c>
-      <c r="B3" s="16">
+      <c r="B3" s="17">
         <f>x4_scale*B2</f>
         <v/>
       </c>
-      <c r="C3" s="16">
+      <c r="C3" s="17">
         <f>x4_scale*C2</f>
         <v/>
       </c>
-      <c r="D3" s="16">
+      <c r="D3" s="17">
         <f>x4_scale*D2</f>
         <v/>
       </c>
@@ -2697,15 +2701,15 @@
           <t>Середнє usage, будівель на клієнта</t>
         </is>
       </c>
-      <c r="B4" s="16">
+      <c r="B4" s="17">
         <f>x4_mix_B*x4_use_B+x4_mix_S*x4_use_S+x4_mix_P*x4_use_P</f>
         <v/>
       </c>
-      <c r="C4" s="16">
+      <c r="C4" s="17">
         <f>x4_mix_B*x4_use_B+x4_mix_S*x4_use_S+x4_mix_P*x4_use_P</f>
         <v/>
       </c>
-      <c r="D4" s="16">
+      <c r="D4" s="17">
         <f>x4_mix_B*x4_use_B+x4_mix_S*x4_use_S+x4_mix_P*x4_use_P</f>
         <v/>
       </c>
@@ -2716,15 +2720,15 @@
           <t>Платні клієнти</t>
         </is>
       </c>
-      <c r="B5" s="16">
+      <c r="B5" s="17">
         <f>B3/B4</f>
         <v/>
       </c>
-      <c r="C5" s="16">
+      <c r="C5" s="17">
         <f>C3/C4</f>
         <v/>
       </c>
-      <c r="D5" s="16">
+      <c r="D5" s="17">
         <f>D3/D4</f>
         <v/>
       </c>
@@ -2735,15 +2739,15 @@
           <t>Клієнти Basic</t>
         </is>
       </c>
-      <c r="B6" s="16">
+      <c r="B6" s="17">
         <f>B5*x4_mix_B</f>
         <v/>
       </c>
-      <c r="C6" s="16">
+      <c r="C6" s="17">
         <f>C5*x4_mix_B</f>
         <v/>
       </c>
-      <c r="D6" s="16">
+      <c r="D6" s="17">
         <f>D5*x4_mix_B</f>
         <v/>
       </c>
@@ -2754,15 +2758,15 @@
           <t>Клієнти Standard</t>
         </is>
       </c>
-      <c r="B7" s="16">
+      <c r="B7" s="17">
         <f>B5*x4_mix_S</f>
         <v/>
       </c>
-      <c r="C7" s="16">
+      <c r="C7" s="17">
         <f>C5*x4_mix_S</f>
         <v/>
       </c>
-      <c r="D7" s="16">
+      <c r="D7" s="17">
         <f>D5*x4_mix_S</f>
         <v/>
       </c>
@@ -2773,15 +2777,15 @@
           <t>Клієнти Pro</t>
         </is>
       </c>
-      <c r="B8" s="16">
+      <c r="B8" s="17">
         <f>B5*x4_mix_P</f>
         <v/>
       </c>
-      <c r="C8" s="16">
+      <c r="C8" s="17">
         <f>C5*x4_mix_P</f>
         <v/>
       </c>
-      <c r="D8" s="16">
+      <c r="D8" s="17">
         <f>D5*x4_mix_P</f>
         <v/>
       </c>
@@ -2792,15 +2796,15 @@
           <t>Revenue: базові платежі</t>
         </is>
       </c>
-      <c r="B9" s="13">
+      <c r="B9" s="14">
         <f>B6*x4_base_B+B7*x4_base_S+B8*x4_base_P</f>
         <v/>
       </c>
-      <c r="C9" s="13">
+      <c r="C9" s="14">
         <f>C6*x4_base_B+C7*x4_base_S+C8*x4_base_P</f>
         <v/>
       </c>
-      <c r="D9" s="13">
+      <c r="D9" s="14">
         <f>D6*x4_base_B+D7*x4_base_S+D8*x4_base_P</f>
         <v/>
       </c>
@@ -2811,15 +2815,15 @@
           <t>Revenue: будівлі (usage)</t>
         </is>
       </c>
-      <c r="B10" s="13">
+      <c r="B10" s="14">
         <f>B6*x4_use_B*x4_pb_B+B7*x4_use_S*x4_pb_S+B8*x4_use_P*x4_pb_P</f>
         <v/>
       </c>
-      <c r="C10" s="13">
+      <c r="C10" s="14">
         <f>C6*x4_use_B*x4_pb_B+C7*x4_use_S*x4_pb_S+C8*x4_use_P*x4_pb_P</f>
         <v/>
       </c>
-      <c r="D10" s="13">
+      <c r="D10" s="14">
         <f>D6*x4_use_B*x4_pb_B+D7*x4_use_S*x4_pb_S+D8*x4_use_P*x4_pb_P</f>
         <v/>
       </c>
@@ -2830,15 +2834,15 @@
           <t>Будівлі з high usage</t>
         </is>
       </c>
-      <c r="B11" s="16">
+      <c r="B11" s="17">
         <f>B3*x4_high_share</f>
         <v/>
       </c>
-      <c r="C11" s="16">
+      <c r="C11" s="17">
         <f>C3*x4_high_share</f>
         <v/>
       </c>
-      <c r="D11" s="16">
+      <c r="D11" s="17">
         <f>D3*x4_high_share</f>
         <v/>
       </c>
@@ -2849,15 +2853,15 @@
           <t>Revenue: overage</t>
         </is>
       </c>
-      <c r="B12" s="13">
+      <c r="B12" s="14">
         <f>B11*x4_over</f>
         <v/>
       </c>
-      <c r="C12" s="13">
+      <c r="C12" s="14">
         <f>C11*x4_over</f>
         <v/>
       </c>
-      <c r="D12" s="13">
+      <c r="D12" s="14">
         <f>D11*x4_over</f>
         <v/>
       </c>
@@ -2868,15 +2872,15 @@
           <t>Revenue</t>
         </is>
       </c>
-      <c r="B13" s="13">
+      <c r="B13" s="14">
         <f>B9+B10+B12</f>
         <v/>
       </c>
-      <c r="C13" s="13">
+      <c r="C13" s="14">
         <f>C9+C10+C12</f>
         <v/>
       </c>
-      <c r="D13" s="13">
+      <c r="D13" s="14">
         <f>D9+D10+D12</f>
         <v/>
       </c>
@@ -2887,15 +2891,15 @@
           <t>COGS: база клієнтів</t>
         </is>
       </c>
-      <c r="B14" s="13">
+      <c r="B14" s="14">
         <f>B6*x4_cc_B+B7*x4_cc_S+B8*x4_cc_P</f>
         <v/>
       </c>
-      <c r="C14" s="13">
+      <c r="C14" s="14">
         <f>C6*x4_cc_B+C7*x4_cc_S+C8*x4_cc_P</f>
         <v/>
       </c>
-      <c r="D14" s="13">
+      <c r="D14" s="14">
         <f>D6*x4_cc_B+D7*x4_cc_S+D8*x4_cc_P</f>
         <v/>
       </c>
@@ -2906,15 +2910,15 @@
           <t>COGS: будівлі</t>
         </is>
       </c>
-      <c r="B15" s="13">
+      <c r="B15" s="14">
         <f>(B3-B11)*x4_cogs+B11*x4_cogs_high</f>
         <v/>
       </c>
-      <c r="C15" s="13">
+      <c r="C15" s="14">
         <f>(C3-C11)*x4_cogs+C11*x4_cogs_high</f>
         <v/>
       </c>
-      <c r="D15" s="13">
+      <c r="D15" s="14">
         <f>(D3-D11)*x4_cogs+D11*x4_cogs_high</f>
         <v/>
       </c>
@@ -2925,15 +2929,15 @@
           <t>COGS</t>
         </is>
       </c>
-      <c r="B16" s="13">
+      <c r="B16" s="14">
         <f>B14+B15</f>
         <v/>
       </c>
-      <c r="C16" s="13">
+      <c r="C16" s="14">
         <f>C14+C15</f>
         <v/>
       </c>
-      <c r="D16" s="13">
+      <c r="D16" s="14">
         <f>D14+D15</f>
         <v/>
       </c>
@@ -2944,15 +2948,15 @@
           <t>Gross profit</t>
         </is>
       </c>
-      <c r="B17" s="13">
+      <c r="B17" s="14">
         <f>B13-B16</f>
         <v/>
       </c>
-      <c r="C17" s="13">
+      <c r="C17" s="14">
         <f>C13-C16</f>
         <v/>
       </c>
-      <c r="D17" s="13">
+      <c r="D17" s="14">
         <f>D13-D16</f>
         <v/>
       </c>
@@ -2963,15 +2967,15 @@
           <t>Gross margin</t>
         </is>
       </c>
-      <c r="B18" s="14">
+      <c r="B18" s="15">
         <f>B17/B13</f>
         <v/>
       </c>
-      <c r="C18" s="14">
+      <c r="C18" s="15">
         <f>C17/C13</f>
         <v/>
       </c>
-      <c r="D18" s="14">
+      <c r="D18" s="15">
         <f>D17/D13</f>
         <v/>
       </c>
@@ -2982,15 +2986,15 @@
           <t>ARPA, EUR на клієнта</t>
         </is>
       </c>
-      <c r="B19" s="13">
+      <c r="B19" s="14">
         <f>B13/B5</f>
         <v/>
       </c>
-      <c r="C19" s="13">
+      <c r="C19" s="14">
         <f>C13/C5</f>
         <v/>
       </c>
-      <c r="D19" s="13">
+      <c r="D19" s="14">
         <f>D13/D5</f>
         <v/>
       </c>
@@ -3001,15 +3005,15 @@
           <t>Revenue на будівлю</t>
         </is>
       </c>
-      <c r="B20" s="13">
+      <c r="B20" s="14">
         <f>B13/B3</f>
         <v/>
       </c>
-      <c r="C20" s="13">
+      <c r="C20" s="14">
         <f>C13/C3</f>
         <v/>
       </c>
-      <c r="D20" s="13">
+      <c r="D20" s="14">
         <f>D13/D3</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
Lab 4 review fixes: expected COGS with unstable buildings, mix weighted margin, grace month effect, A8 and A9 assumptions, wider tariff grid
</commit_message>
<xml_diff>
--- a/lab4/out/lab4_pricing.xlsx
+++ b/lab4/out/lab4_pricing.xlsx
@@ -33,10 +33,11 @@
     <definedName name="x4_value">'Параметри ЛР4'!$C$17</definedName>
     <definedName name="x4_energy">'Параметри ЛР4'!$C$18</definedName>
     <definedName name="x4_gain">'Параметри ЛР4'!$C$19</definedName>
-    <definedName name="x4_cogs">'Параметри ЛР4'!$C$21</definedName>
-    <definedName name="x4_cogs_high">'Параметри ЛР4'!$C$22</definedName>
-    <definedName name="x4_over">'Параметри ЛР4'!$C$23</definedName>
-    <definedName name="x4_floor_unit">'Параметри ЛР4'!$C$24</definedName>
+    <definedName name="x4_episode">'Параметри ЛР4'!$C$20</definedName>
+    <definedName name="x4_cogs">'Параметри ЛР4'!$C$22</definedName>
+    <definedName name="x4_cogs_high">'Параметри ЛР4'!$C$23</definedName>
+    <definedName name="x4_over">'Параметри ЛР4'!$C$24</definedName>
+    <definedName name="x4_floor_unit">'Параметри ЛР4'!$C$25</definedName>
     <definedName name="x4_mix_B">'Тарифи'!$C$5</definedName>
     <definedName name="x4_use_B">'Тарифи'!$C$6</definedName>
     <definedName name="x4_base_B">'Тарифи'!$C$2</definedName>
@@ -126,7 +127,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
@@ -172,6 +173,12 @@
     </xf>
     <xf numFmtId="165" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="10" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="9" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="top" wrapText="1"/>
@@ -735,7 +742,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F24"/>
+  <dimension ref="A1:F25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1319,56 +1326,56 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="2" t="n"/>
-      <c r="B20" s="2" t="n"/>
-      <c r="C20" s="2" t="n"/>
-      <c r="D20" s="2" t="n"/>
-      <c r="E20" s="2" t="n"/>
-      <c r="F20" s="2" t="n"/>
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>x4_episode</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>Тривалість епізоду нестабільності</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>міс.</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>П</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>A9</t>
+        </is>
+      </c>
     </row>
     <row r="21">
-      <c r="A21" s="2" t="inlineStr">
-        <is>
-          <t>x4_cogs</t>
-        </is>
-      </c>
-      <c r="B21" s="2" t="inlineStr">
-        <is>
-          <t>COGS на будівлю з компонентів ЛР № 1</t>
-        </is>
-      </c>
-      <c r="C21" s="5">
-        <f>x4_readings+x4_sim+x4_sms_cost*x4_sms_typ+x4_sup_h*x4_sup_rate</f>
-        <v/>
-      </c>
-      <c r="D21" s="2" t="inlineStr">
-        <is>
-          <t>EUR/буд./міс.</t>
-        </is>
-      </c>
-      <c r="E21" s="2" t="inlineStr">
-        <is>
-          <t>Р</t>
-        </is>
-      </c>
-      <c r="F21" s="6">
-        <f>IF(ABS(C21-x4_cogs_var)&lt;0.001,"збігається з варіантом","розбіжність")</f>
-        <v/>
-      </c>
+      <c r="A21" s="2" t="n"/>
+      <c r="B21" s="2" t="n"/>
+      <c r="C21" s="2" t="n"/>
+      <c r="D21" s="2" t="n"/>
+      <c r="E21" s="2" t="n"/>
+      <c r="F21" s="2" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>x4_cogs_high</t>
+          <t>x4_cogs</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>COGS будівлі з high usage</t>
+          <t>COGS на будівлю з компонентів ЛР № 1</t>
         </is>
       </c>
       <c r="C22" s="5">
-        <f>x4_cogs+(x4_sms_high-x4_sms_typ)*x4_sms_cost+(x4_sup_high-x4_sup_h)*x4_sup_rate</f>
+        <f>x4_readings+x4_sim+x4_sms_cost*x4_sms_typ+x4_sup_h*x4_sup_rate</f>
         <v/>
       </c>
       <c r="D22" s="2" t="inlineStr">
@@ -1381,25 +1388,24 @@
           <t>Р</t>
         </is>
       </c>
-      <c r="F22" s="2" t="inlineStr">
-        <is>
-          <t>A3</t>
-        </is>
+      <c r="F22" s="6">
+        <f>IF(ABS(C22-x4_cogs_var)&lt;0.001,"збігається з варіантом","розбіжність")</f>
+        <v/>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>x4_over</t>
+          <t>x4_cogs_high</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>Overage з будівлі з high usage</t>
+          <t>COGS будівлі з high usage</t>
         </is>
       </c>
       <c r="C23" s="5">
-        <f>x4_fee+MAX(x4_sms_high-x4_sms_incl,0)*x4_sms_price</f>
+        <f>x4_cogs+(x4_sms_high-x4_sms_typ)*x4_sms_cost+(x4_sup_high-x4_sup_h)*x4_sup_rate</f>
         <v/>
       </c>
       <c r="D23" s="2" t="inlineStr">
@@ -1414,36 +1420,67 @@
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>доплата + SMS понад ліміт</t>
+          <t>A3</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
+          <t>x4_over</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>Overage з будівлі з high usage</t>
+        </is>
+      </c>
+      <c r="C24" s="5">
+        <f>x4_fee+MAX(x4_sms_high-x4_sms_incl,0)*x4_sms_price</f>
+        <v/>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>EUR/буд./міс.</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>Р</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>доплата + SMS понад ліміт</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
           <t>x4_floor_unit</t>
         </is>
       </c>
-      <c r="B24" s="2" t="inlineStr">
+      <c r="B25" s="2" t="inlineStr">
         <is>
           <t>Floor price на будівлю</t>
         </is>
       </c>
-      <c r="C24" s="5">
+      <c r="C25" s="5">
         <f>x4_cogs_var/(1-x4_gm)</f>
         <v/>
       </c>
-      <c r="D24" s="2" t="inlineStr">
+      <c r="D25" s="2" t="inlineStr">
         <is>
           <t>EUR/буд./міс.</t>
         </is>
       </c>
-      <c r="E24" s="2" t="inlineStr">
+      <c r="E25" s="2" t="inlineStr">
         <is>
           <t>Р</t>
         </is>
       </c>
-      <c r="F24" s="2" t="inlineStr">
+      <c r="F25" s="2" t="inlineStr">
         <is>
           <t>COGS / (1 − GM)</t>
         </is>
@@ -1461,7 +1498,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1684,6 +1721,60 @@
       <c r="E8" s="2" t="inlineStr">
         <is>
           <t>Revenue, COGS</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>A8</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Готовність платити за будівлю</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>130...135 EUR на місяць за будівлю, не більше 15% цінності 900 EUR</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>П: гіпотеза A2 ЛР № 1, листами про намір не перевірена</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>Revenue, GM</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>A9</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Стаціонарний стан доплати за нестабільний облік</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>у сценаріях Y3 усі будівлі зі статусом «нестабільний облік» уже пройшли 2 місяці спостереження і 1 пільговий місяць; епізод нестабільності триває 12 місяців</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>П: спрощення; вплив від 1 до 3 неоплачених місяців наведено в додатку</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>Revenue overage, GM</t>
         </is>
       </c>
     </row>
@@ -1877,7 +1968,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E23"/>
+  <dimension ref="A1:E32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -2328,50 +2419,204 @@
         <v/>
       </c>
     </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>Очікуваний COGS будівлі з A3, EUR</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>0,9 × 16 + 0,1 × 30,88</t>
+        </is>
+      </c>
+      <c r="C20" s="14">
+        <f>(1-x4_high_share)*x4_cogs+x4_high_share*x4_cogs_high</f>
+        <v/>
+      </c>
+      <c r="D20" s="14">
+        <f>(1-x4_high_share)*x4_cogs+x4_high_share*x4_cogs_high</f>
+        <v/>
+      </c>
+      <c r="E20" s="14">
+        <f>(1-x4_high_share)*x4_cogs+x4_high_share*x4_cogs_high</f>
+        <v/>
+      </c>
+    </row>
     <row r="21">
-      <c r="A21" s="1" t="inlineStr">
-        <is>
-          <t>Перевірка формули floor</t>
-        </is>
-      </c>
-      <c r="B21" s="1" t="inlineStr">
-        <is>
-          <t>Значення, EUR</t>
-        </is>
-      </c>
-      <c r="C21" s="1" t="inlineStr">
-        <is>
-          <t>GM</t>
-        </is>
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>Очікуваний COGS клієнта з A3, EUR/міс.</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>COGS бази + usage × 17,49</t>
+        </is>
+      </c>
+      <c r="C21" s="14">
+        <f>C8+C6*C20</f>
+        <v/>
+      </c>
+      <c r="D21" s="14">
+        <f>D8+D6*D20</f>
+        <v/>
+      </c>
+      <c r="E21" s="14">
+        <f>E8+E6*E20</f>
+        <v/>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Правильно: COGS / (1 − GM)</t>
-        </is>
-      </c>
-      <c r="B22" s="5">
-        <f>x4_cogs_var/(1-x4_gm)</f>
-        <v/>
-      </c>
-      <c r="C22" s="15">
-        <f>(B22-x4_cogs_var)/B22</f>
+          <t>Очікуваний overage з A3, EUR/міс.</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>usage × 0,10 × 55</t>
+        </is>
+      </c>
+      <c r="C22" s="14">
+        <f>C6*x4_high_share*x4_over</f>
+        <v/>
+      </c>
+      <c r="D22" s="14">
+        <f>D6*x4_high_share*x4_over</f>
+        <v/>
+      </c>
+      <c r="E22" s="14">
+        <f>E6*x4_high_share*x4_over</f>
         <v/>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
+          <t>Очікуваний рахунок з A3, EUR/міс.</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>рахунок + overage</t>
+        </is>
+      </c>
+      <c r="C23" s="14">
+        <f>C9+C22</f>
+        <v/>
+      </c>
+      <c r="D23" s="14">
+        <f>D9+D22</f>
+        <v/>
+      </c>
+      <c r="E23" s="14">
+        <f>E9+E22</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>Gross margin з A3</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>(Revenue − COGS) / Revenue</t>
+        </is>
+      </c>
+      <c r="C24" s="15">
+        <f>(C23-C21)/C23</f>
+        <v/>
+      </c>
+      <c r="D24" s="15">
+        <f>(D23-D21)/D23</f>
+        <v/>
+      </c>
+      <c r="E24" s="15">
+        <f>(E23-E21)/E23</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="1" t="inlineStr">
+        <is>
+          <t>Перевірка формули floor</t>
+        </is>
+      </c>
+      <c r="B26" s="1" t="inlineStr">
+        <is>
+          <t>Значення, EUR</t>
+        </is>
+      </c>
+      <c r="C26" s="1" t="inlineStr">
+        <is>
+          <t>GM</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>Правильно: COGS / (1 − GM)</t>
+        </is>
+      </c>
+      <c r="B27" s="5">
+        <f>x4_cogs_var/(1-x4_gm)</f>
+        <v/>
+      </c>
+      <c r="C27" s="15">
+        <f>(B27-x4_cogs_var)/B27</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
           <t>Помилково: COGS × (1 + GM)</t>
         </is>
       </c>
-      <c r="B23" s="5">
+      <c r="B28" s="5">
         <f>x4_cogs_var*(1+x4_gm)</f>
         <v/>
       </c>
-      <c r="C23" s="15">
-        <f>(B23-x4_cogs_var)/B23</f>
+      <c r="C28" s="15">
+        <f>(B28-x4_cogs_var)/B28</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="1" t="inlineStr">
+        <is>
+          <t>Зважена за A1 gross margin</t>
+        </is>
+      </c>
+      <c r="B30" s="1" t="inlineStr">
+        <is>
+          <t>Значення</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>Типова будівля, без A3</t>
+        </is>
+      </c>
+      <c r="B31" s="16">
+        <f>(x4_mix_B*(C9-C10)+x4_mix_S*(D9-D10)+x4_mix_P*(E9-E10))/(x4_mix_B*C9+x4_mix_S*D9+x4_mix_P*E9)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>З урахуванням A3, дорівнює GM сценаріїв</t>
+        </is>
+      </c>
+      <c r="B32" s="16">
+        <f>(x4_mix_B*(C23-C21)+x4_mix_S*(D23-D21)+x4_mix_P*(E23-E21))/(x4_mix_B*C23+x4_mix_S*D23+x4_mix_P*E23)</f>
         <v/>
       </c>
     </row>
@@ -2387,14 +2632,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:F17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="34" customWidth="1" min="1" max="1"/>
-    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="38" customWidth="1" min="1" max="1"/>
+    <col width="31" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2614,6 +2860,170 @@
       </c>
       <c r="E10" s="14">
         <f>IF(E8&gt;=x4_gm,"так","ні")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="1" t="inlineStr">
+        <is>
+          <t>Неоплачених місяців з 12 (A9)</t>
+        </is>
+      </c>
+      <c r="B12" s="1" t="inlineStr">
+        <is>
+          <t>Формула</t>
+        </is>
+      </c>
+      <c r="C12" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="D12" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="E12" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="F12" s="17" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Overage, базовий сценарій, EUR</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>overage − буд. high × 50 × m / 12</t>
+        </is>
+      </c>
+      <c r="C13" s="14">
+        <f>'Сценарії'!$C$12-'Сценарії'!$C$11*x4_fee*C12/x4_episode</f>
+        <v/>
+      </c>
+      <c r="D13" s="14">
+        <f>'Сценарії'!$C$12-'Сценарії'!$C$11*x4_fee*D12/x4_episode</f>
+        <v/>
+      </c>
+      <c r="E13" s="14">
+        <f>'Сценарії'!$C$12-'Сценарії'!$C$11*x4_fee*E12/x4_episode</f>
+        <v/>
+      </c>
+      <c r="F13" s="14">
+        <f>'Сценарії'!$C$12-'Сценарії'!$C$11*x4_fee*F12/x4_episode</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Revenue, базовий сценарій, EUR</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Revenue − та сама втрата</t>
+        </is>
+      </c>
+      <c r="C14" s="14">
+        <f>'Сценарії'!$C$13-'Сценарії'!$C$11*x4_fee*C12/x4_episode</f>
+        <v/>
+      </c>
+      <c r="D14" s="14">
+        <f>'Сценарії'!$C$13-'Сценарії'!$C$11*x4_fee*D12/x4_episode</f>
+        <v/>
+      </c>
+      <c r="E14" s="14">
+        <f>'Сценарії'!$C$13-'Сценарії'!$C$11*x4_fee*E12/x4_episode</f>
+        <v/>
+      </c>
+      <c r="F14" s="14">
+        <f>'Сценарії'!$C$13-'Сценарії'!$C$11*x4_fee*F12/x4_episode</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Gross margin, базовий сценарій</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>(Revenue − COGS) / Revenue</t>
+        </is>
+      </c>
+      <c r="C15" s="15">
+        <f>(C14-'Сценарії'!$C$16)/C14</f>
+        <v/>
+      </c>
+      <c r="D15" s="15">
+        <f>(D14-'Сценарії'!$C$16)/D14</f>
+        <v/>
+      </c>
+      <c r="E15" s="15">
+        <f>(E14-'Сценарії'!$C$16)/E14</f>
+        <v/>
+      </c>
+      <c r="F15" s="15">
+        <f>(F14-'Сценарії'!$C$16)/F14</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>GM Pro, 20 буд., неоплачений місяць</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>рахунок без доплати</t>
+        </is>
+      </c>
+      <c r="C16" s="15">
+        <f>($E$7-$E$2*x4_fee-$E$4)/($E$7-$E$2*x4_fee)</f>
+        <v/>
+      </c>
+      <c r="D16" s="15">
+        <f>($E$7-$E$2*x4_fee-$E$4)/($E$7-$E$2*x4_fee)</f>
+        <v/>
+      </c>
+      <c r="E16" s="15">
+        <f>($E$7-$E$2*x4_fee-$E$4)/($E$7-$E$2*x4_fee)</f>
+        <v/>
+      </c>
+      <c r="F16" s="15">
+        <f>($E$7-$E$2*x4_fee-$E$4)/($E$7-$E$2*x4_fee)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>GM Pro, 20 буд., за 12 місяців</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>зважено за місяцями</t>
+        </is>
+      </c>
+      <c r="C17" s="15">
+        <f>($E$7*(x4_episode-C12)+($E$7-$E$2*x4_fee)*C12-x4_episode*$E$4)/($E$7*(x4_episode-C12)+($E$7-$E$2*x4_fee)*C12)</f>
+        <v/>
+      </c>
+      <c r="D17" s="15">
+        <f>($E$7*(x4_episode-D12)+($E$7-$E$2*x4_fee)*D12-x4_episode*$E$4)/($E$7*(x4_episode-D12)+($E$7-$E$2*x4_fee)*D12)</f>
+        <v/>
+      </c>
+      <c r="E17" s="15">
+        <f>($E$7*(x4_episode-E12)+($E$7-$E$2*x4_fee)*E12-x4_episode*$E$4)/($E$7*(x4_episode-E12)+($E$7-$E$2*x4_fee)*E12)</f>
+        <v/>
+      </c>
+      <c r="F17" s="15">
+        <f>($E$7*(x4_episode-F12)+($E$7-$E$2*x4_fee)*F12-x4_episode*$E$4)/($E$7*(x4_episode-F12)+($E$7-$E$2*x4_fee)*F12)</f>
         <v/>
       </c>
     </row>
@@ -2666,13 +3076,13 @@
           <t>Коефіцієнт масштабу</t>
         </is>
       </c>
-      <c r="B2" s="16" t="n">
+      <c r="B2" s="18" t="n">
         <v>0.7</v>
       </c>
-      <c r="C2" s="16" t="n">
+      <c r="C2" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="D2" s="16" t="n">
+      <c r="D2" s="18" t="n">
         <v>1.4</v>
       </c>
     </row>
@@ -2682,15 +3092,15 @@
           <t>Платні будівлі (billable units)</t>
         </is>
       </c>
-      <c r="B3" s="17">
+      <c r="B3" s="19">
         <f>x4_scale*B2</f>
         <v/>
       </c>
-      <c r="C3" s="17">
+      <c r="C3" s="19">
         <f>x4_scale*C2</f>
         <v/>
       </c>
-      <c r="D3" s="17">
+      <c r="D3" s="19">
         <f>x4_scale*D2</f>
         <v/>
       </c>
@@ -2701,15 +3111,15 @@
           <t>Середнє usage, будівель на клієнта</t>
         </is>
       </c>
-      <c r="B4" s="17">
+      <c r="B4" s="19">
         <f>x4_mix_B*x4_use_B+x4_mix_S*x4_use_S+x4_mix_P*x4_use_P</f>
         <v/>
       </c>
-      <c r="C4" s="17">
+      <c r="C4" s="19">
         <f>x4_mix_B*x4_use_B+x4_mix_S*x4_use_S+x4_mix_P*x4_use_P</f>
         <v/>
       </c>
-      <c r="D4" s="17">
+      <c r="D4" s="19">
         <f>x4_mix_B*x4_use_B+x4_mix_S*x4_use_S+x4_mix_P*x4_use_P</f>
         <v/>
       </c>
@@ -2720,15 +3130,15 @@
           <t>Платні клієнти</t>
         </is>
       </c>
-      <c r="B5" s="17">
+      <c r="B5" s="19">
         <f>B3/B4</f>
         <v/>
       </c>
-      <c r="C5" s="17">
+      <c r="C5" s="19">
         <f>C3/C4</f>
         <v/>
       </c>
-      <c r="D5" s="17">
+      <c r="D5" s="19">
         <f>D3/D4</f>
         <v/>
       </c>
@@ -2739,15 +3149,15 @@
           <t>Клієнти Basic</t>
         </is>
       </c>
-      <c r="B6" s="17">
+      <c r="B6" s="19">
         <f>B5*x4_mix_B</f>
         <v/>
       </c>
-      <c r="C6" s="17">
+      <c r="C6" s="19">
         <f>C5*x4_mix_B</f>
         <v/>
       </c>
-      <c r="D6" s="17">
+      <c r="D6" s="19">
         <f>D5*x4_mix_B</f>
         <v/>
       </c>
@@ -2758,15 +3168,15 @@
           <t>Клієнти Standard</t>
         </is>
       </c>
-      <c r="B7" s="17">
+      <c r="B7" s="19">
         <f>B5*x4_mix_S</f>
         <v/>
       </c>
-      <c r="C7" s="17">
+      <c r="C7" s="19">
         <f>C5*x4_mix_S</f>
         <v/>
       </c>
-      <c r="D7" s="17">
+      <c r="D7" s="19">
         <f>D5*x4_mix_S</f>
         <v/>
       </c>
@@ -2777,15 +3187,15 @@
           <t>Клієнти Pro</t>
         </is>
       </c>
-      <c r="B8" s="17">
+      <c r="B8" s="19">
         <f>B5*x4_mix_P</f>
         <v/>
       </c>
-      <c r="C8" s="17">
+      <c r="C8" s="19">
         <f>C5*x4_mix_P</f>
         <v/>
       </c>
-      <c r="D8" s="17">
+      <c r="D8" s="19">
         <f>D5*x4_mix_P</f>
         <v/>
       </c>
@@ -2834,15 +3244,15 @@
           <t>Будівлі з high usage</t>
         </is>
       </c>
-      <c r="B11" s="17">
+      <c r="B11" s="19">
         <f>B3*x4_high_share</f>
         <v/>
       </c>
-      <c r="C11" s="17">
+      <c r="C11" s="19">
         <f>C3*x4_high_share</f>
         <v/>
       </c>
-      <c r="D11" s="17">
+      <c r="D11" s="19">
         <f>D3*x4_high_share</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
Lab 4 consistency: A8 states lab 1 letter of intent threshold revised from 130 to 135 EUR with reason, scale 85 read as Y3 monthly average as in lab 3
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/lab4/out/lab4_pricing.xlsx
+++ b/lab4/out/lab4_pricing.xlsx
@@ -1737,12 +1737,12 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>130...135 EUR на місяць за будівлю, не більше 15% цінності 900 EUR</t>
+          <t>130...135 EUR на місяць за будівлю, не більше 15% цінності 900 EUR; тест: не менше 3 листів про намір з 10 інтерв'ю за ціною 135 EUR</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>П: гіпотеза A2 ЛР № 1, листами про намір не перевірена</t>
+          <t>П: гіпотеза A2 ЛР № 1, листами про намір не перевірена; поріг тесту A2 ЛР № 1 переглянуто з 130 до 135 EUR, бо рахунок Basic за 1 будівлю дорівнює 135 EUR</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">

</xml_diff>